<commit_message>
improved scan ui to allow for patient field edits and cleaner display of scan results
</commit_message>
<xml_diff>
--- a/data/mock_patients.xlsx
+++ b/data/mock_patients.xlsx
@@ -516,7 +516,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>(539)776-8542x1764</t>
+          <t>(539)776-8542</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -541,7 +541,7 @@
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>2026-05-27T13:04:12.308635</t>
+          <t>2026-05-28T11:39:31.683341</t>
         </is>
       </c>
     </row>
@@ -5625,7 +5625,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F75"/>
+  <dimension ref="A1:F91"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7672,6 +7672,454 @@
         </is>
       </c>
     </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>2026-05-28T11:19:02.427096</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>6ec2416d</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr"/>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>SCAN_LOOKUP</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>streamlit_ui</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>scan_tab</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>2026-05-28T11:20:24.564625</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>6ec2416d</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr"/>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>SCAN_LOOKUP</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>streamlit_ui</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>scan_tab</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>2026-05-28T11:20:24.704201</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>5da3568e</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr"/>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>DIRECTORY_SEARCH</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>streamlit_ui</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>arm</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>2026-05-28T11:20:27.137944</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>6ec2416d</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr"/>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>SCAN_LOOKUP</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>streamlit_ui</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>scan_tab</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>2026-05-28T11:20:27.227240</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>47843209</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr"/>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>DIRECTORY_SEARCH</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>streamlit_ui</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>arman</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>2026-05-28T11:20:31.352908</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>6ec2416d</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr"/>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>SCAN_LOOKUP</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>streamlit_ui</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>scan_tab</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>2026-05-28T11:20:31.440252</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>47843209</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr"/>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>DIRECTORY_SEARCH</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>streamlit_ui</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>armanalay</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>2026-05-28T11:20:36.130166</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>6ec2416d</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr"/>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>SCAN_LOOKUP</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>streamlit_ui</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>scan_tab</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>2026-05-28T11:20:36.219930</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>47843209</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr"/>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>DIRECTORY_SEARCH</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>streamlit_ui</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>sam</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>2026-05-28T11:39:07.148717</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>6ec2416d</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr"/>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>SCAN_LOOKUP</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>streamlit_ui</t>
+        </is>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>scan_tab</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>2026-05-28T11:39:15.533931</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>6ec2416d</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr"/>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>SCAN_LOOKUP</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>streamlit_ui</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>scan_tab</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>2026-05-28T11:39:18.236045</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>6ec2416d</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr"/>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>SCAN_LOOKUP</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>streamlit_ui</t>
+        </is>
+      </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>scan_tab</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>2026-05-28T11:39:26.958719</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>6ec2416d</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr"/>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>SCAN_LOOKUP</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>streamlit_ui</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>scan_tab</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>2026-05-28T11:39:29.311454</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>6ec2416d</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr"/>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>SCAN_LOOKUP</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>streamlit_ui</t>
+        </is>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>scan_tab</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>2026-05-28T11:39:31.590989</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>6ec2416d</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr"/>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>SCAN_LOOKUP</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>streamlit_ui</t>
+        </is>
+      </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>scan_tab</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>2026-05-28T11:39:31.775208</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>6ec2416d</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr"/>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>SCAN_LOOKUP</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>streamlit_ui</t>
+        </is>
+      </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>scan_tab</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>